<commit_message>
Umbau auf BM64 zur Freigabe
</commit_message>
<xml_diff>
--- a/BOM/20220322 BOM TeKaDe Baseboard 5VEXT BM64.xlsx
+++ b/BOM/20220322 BOM TeKaDe Baseboard 5VEXT BM64.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IngBuero\Projekte_Kunden\2021_TeKaDeRevival\PCB\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IngBuero\Projekte_Kunden\2021_TeKaDeRevival\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F1CC417-0980-4662-ABF0-90F1C81BB219}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7854631-05DF-4736-B561-3A64298D75F5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11957" xr2:uid="{261E8F2A-9F01-4E4B-AED6-14B6866C8B8C}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11960" xr2:uid="{261E8F2A-9F01-4E4B-AED6-14B6866C8B8C}"/>
   </bookViews>
   <sheets>
     <sheet name="Vollständig" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="788" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="792" uniqueCount="371">
   <si>
     <t>Gesamtpreis</t>
   </si>
@@ -1136,6 +1136,9 @@
   </si>
   <si>
     <t xml:space="preserve">BM64 BT Module </t>
+  </si>
+  <si>
+    <t>J9</t>
   </si>
 </sst>
 </file>
@@ -1629,28 +1632,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABABC861-D339-4CAE-9A46-3EF0A1CCE7F9}">
-  <dimension ref="A1:Z94"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" outlineLevelCol="1" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:Z95"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.35" outlineLevelCol="1" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="4.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.3828125" customWidth="1"/>
-    <col min="3" max="3" width="31.69140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.3828125" customWidth="1"/>
-    <col min="5" max="5" width="17.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.3515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.3515625" customWidth="1"/>
+    <col min="3" max="3" width="31.703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.3515625" customWidth="1"/>
+    <col min="5" max="5" width="17.05859375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.61328125" customWidth="1"/>
-    <col min="8" max="8" width="15.4609375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.3828125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="2.84375" style="4" customWidth="1" outlineLevel="1"/>
-    <col min="11" max="11" width="22.921875" bestFit="1" customWidth="1" outlineLevel="1"/>
+    <col min="7" max="7" width="12.5859375" customWidth="1"/>
+    <col min="8" max="8" width="15.46875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.3515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="2.8203125" style="4" customWidth="1" outlineLevel="1"/>
+    <col min="11" max="11" width="22.9375" bestFit="1" customWidth="1" outlineLevel="1"/>
     <col min="12" max="12" width="13" bestFit="1" customWidth="1" outlineLevel="1"/>
     <col min="13" max="14" width="11" customWidth="1" outlineLevel="1"/>
-    <col min="15" max="16" width="10.921875" customWidth="1" outlineLevel="1"/>
-    <col min="17" max="17" width="7.53515625" customWidth="1" outlineLevel="1"/>
-    <col min="18" max="26" width="10.921875" customWidth="1" outlineLevel="1"/>
+    <col min="15" max="16" width="10.9375" customWidth="1" outlineLevel="1"/>
+    <col min="17" max="17" width="7.52734375" customWidth="1" outlineLevel="1"/>
+    <col min="18" max="26" width="10.9375" customWidth="1" outlineLevel="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.5">
       <c r="K1" s="38" t="s">
         <v>4</v>
       </c>
@@ -1662,7 +1665,7 @@
       </c>
       <c r="P1" s="38"/>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -1709,7 +1712,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1755,7 +1758,7 @@
         <v>6.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A4" s="7">
         <v>2</v>
       </c>
@@ -1801,7 +1804,7 @@
       </c>
       <c r="Q4" s="7"/>
     </row>
-    <row r="5" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A5">
         <v>3</v>
       </c>
@@ -1845,7 +1848,7 @@
         <v>0.13200000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A6">
         <v>4</v>
       </c>
@@ -1888,7 +1891,7 @@
         <v>0.70399999999999996</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A7" s="7">
         <v>5</v>
       </c>
@@ -1931,7 +1934,7 @@
         <v>2.1999999999999999E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A8">
         <v>6</v>
       </c>
@@ -1974,7 +1977,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A9">
         <v>7</v>
       </c>
@@ -2017,7 +2020,7 @@
         <v>0.30599999999999999</v>
       </c>
     </row>
-    <row r="10" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A10" s="7">
         <v>8</v>
       </c>
@@ -2063,7 +2066,7 @@
         <v>0.13400000000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A11">
         <v>9</v>
       </c>
@@ -2092,7 +2095,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A12">
         <v>10</v>
       </c>
@@ -2139,7 +2142,7 @@
         <v>3.9E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A13" s="7">
         <v>11</v>
       </c>
@@ -2187,7 +2190,7 @@
       </c>
       <c r="Q13" s="7"/>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A14">
         <v>12</v>
       </c>
@@ -2236,7 +2239,7 @@
       <c r="Q14" s="7"/>
       <c r="R14" s="7"/>
     </row>
-    <row r="15" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A15">
         <v>13</v>
       </c>
@@ -2283,7 +2286,7 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A16" s="7">
         <v>14</v>
       </c>
@@ -2330,7 +2333,7 @@
         <v>6.4000000000000001E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A17">
         <v>15</v>
       </c>
@@ -2377,7 +2380,7 @@
         <v>5.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A18">
         <v>16</v>
       </c>
@@ -2424,7 +2427,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A19" s="7">
         <v>17</v>
       </c>
@@ -2471,7 +2474,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A20">
         <v>18</v>
       </c>
@@ -2518,7 +2521,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:16" s="12" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:16" s="12" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A21">
         <v>19</v>
       </c>
@@ -2566,7 +2569,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A22" s="7">
         <v>20</v>
       </c>
@@ -2613,7 +2616,7 @@
         <v>6.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A23">
         <v>21</v>
       </c>
@@ -2660,7 +2663,7 @@
         <v>1.2E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A24">
         <v>22</v>
       </c>
@@ -2707,7 +2710,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A25" s="7">
         <v>23</v>
       </c>
@@ -2754,7 +2757,7 @@
         <v>1.4E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A26">
         <v>24</v>
       </c>
@@ -2801,7 +2804,7 @@
         <v>2.4E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A27">
         <v>25</v>
       </c>
@@ -2848,7 +2851,7 @@
         <v>5.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="28" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A28" s="7">
         <v>26</v>
       </c>
@@ -2877,7 +2880,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A29">
         <v>27</v>
       </c>
@@ -2905,7 +2908,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A30">
         <v>28</v>
       </c>
@@ -2952,7 +2955,7 @@
         <v>1.2E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A31" s="7">
         <v>29</v>
       </c>
@@ -2999,7 +3002,7 @@
         <v>4.3999999999999997E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A32">
         <v>30</v>
       </c>
@@ -3046,7 +3049,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A33">
         <v>31</v>
       </c>
@@ -3093,7 +3096,7 @@
         <v>4.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A34" s="7">
         <v>32</v>
       </c>
@@ -3140,7 +3143,7 @@
         <v>1.6E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A35">
         <v>33</v>
       </c>
@@ -3187,7 +3190,7 @@
         <v>0.13400000000000001</v>
       </c>
     </row>
-    <row r="36" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A36">
         <v>34</v>
       </c>
@@ -3235,7 +3238,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A37" s="7">
         <v>35</v>
       </c>
@@ -3281,13 +3284,13 @@
         <v>1.04</v>
       </c>
     </row>
-    <row r="38" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.5">
       <c r="M38" s="5"/>
       <c r="N38" s="5"/>
       <c r="O38" s="33"/>
       <c r="P38" s="33"/>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A39">
         <v>36</v>
       </c>
@@ -3331,7 +3334,7 @@
       </c>
       <c r="Q39" s="7"/>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A40">
         <v>37</v>
       </c>
@@ -3379,7 +3382,7 @@
       </c>
       <c r="Q40" s="7"/>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A41">
         <v>38</v>
       </c>
@@ -3425,7 +3428,7 @@
       <c r="Q41" s="7"/>
       <c r="R41" s="35"/>
     </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A42">
         <v>39</v>
       </c>
@@ -3475,7 +3478,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A43">
         <v>40</v>
       </c>
@@ -3521,7 +3524,7 @@
       </c>
       <c r="Q43" s="7"/>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A44">
         <v>41</v>
       </c>
@@ -3567,7 +3570,7 @@
       </c>
       <c r="Q44" s="7"/>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A45">
         <v>42</v>
       </c>
@@ -3613,7 +3616,7 @@
       </c>
       <c r="Q45" s="7"/>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A46">
         <v>43</v>
       </c>
@@ -3660,7 +3663,7 @@
       </c>
       <c r="Q46" s="7"/>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A47">
         <v>44</v>
       </c>
@@ -3704,7 +3707,7 @@
       </c>
       <c r="Q47" s="7"/>
     </row>
-    <row r="48" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A48">
         <v>45</v>
       </c>
@@ -3749,7 +3752,7 @@
       </c>
       <c r="Q48" s="10"/>
     </row>
-    <row r="49" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A49" s="7">
         <v>46</v>
       </c>
@@ -3796,7 +3799,7 @@
       </c>
       <c r="Q49" s="7"/>
     </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A50">
         <v>47</v>
       </c>
@@ -3844,13 +3847,13 @@
       <c r="Q50" s="7"/>
       <c r="R50" s="35"/>
     </row>
-    <row r="51" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.5">
       <c r="M51" s="25"/>
       <c r="N51" s="25"/>
       <c r="O51" s="33"/>
       <c r="P51" s="33"/>
     </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A52">
         <v>48</v>
       </c>
@@ -3896,7 +3899,7 @@
         <v>0.27800000000000002</v>
       </c>
     </row>
-    <row r="53" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A53">
         <v>49</v>
       </c>
@@ -3942,7 +3945,7 @@
         <v>0.27900000000000003</v>
       </c>
     </row>
-    <row r="54" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A54">
         <v>50</v>
       </c>
@@ -3988,7 +3991,7 @@
         <v>0.32700000000000001</v>
       </c>
     </row>
-    <row r="55" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A55">
         <v>51</v>
       </c>
@@ -4035,7 +4038,7 @@
         <v>3.9E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A56">
         <v>52</v>
       </c>
@@ -4080,7 +4083,7 @@
         <v>8.5000000000000006E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A57">
         <v>53</v>
       </c>
@@ -4125,7 +4128,7 @@
         <v>8.5000000000000006E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A58">
         <v>54</v>
       </c>
@@ -4170,7 +4173,7 @@
         <v>8.5000000000000006E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:18" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:18" x14ac:dyDescent="0.5">
       <c r="A59">
         <v>55</v>
       </c>
@@ -4219,7 +4222,7 @@
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A60">
         <v>56</v>
       </c>
@@ -4267,13 +4270,13 @@
         <v>7.8E-2</v>
       </c>
     </row>
-    <row r="61" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.5">
       <c r="M61" s="25"/>
       <c r="N61" s="25"/>
       <c r="O61" s="33"/>
       <c r="P61" s="33"/>
     </row>
-    <row r="62" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A62" s="17">
         <v>57</v>
       </c>
@@ -4320,7 +4323,7 @@
         <v>9.7000000000000003E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A63" s="17">
         <v>58</v>
       </c>
@@ -4365,13 +4368,13 @@
         <v>0.26</v>
       </c>
     </row>
-    <row r="64" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.5">
       <c r="M64" s="25"/>
       <c r="N64" s="25"/>
       <c r="O64" s="33"/>
       <c r="P64" s="33"/>
     </row>
-    <row r="65" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A65" s="17">
         <v>59</v>
       </c>
@@ -4418,7 +4421,7 @@
         <v>0.65600000000000003</v>
       </c>
     </row>
-    <row r="66" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A66" s="17">
         <v>60</v>
       </c>
@@ -4465,13 +4468,13 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="67" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.5">
       <c r="M67" s="25"/>
       <c r="N67" s="25"/>
       <c r="O67" s="33"/>
       <c r="P67" s="33"/>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A68" s="17">
         <v>61</v>
       </c>
@@ -4517,7 +4520,7 @@
         <v>1.24</v>
       </c>
     </row>
-    <row r="69" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A69">
         <v>62</v>
       </c>
@@ -4534,15 +4537,15 @@
       <c r="M69" s="28"/>
       <c r="N69" s="28"/>
       <c r="O69" s="32">
-        <f t="shared" ref="O69:O76" si="4">B69*M69</f>
+        <f t="shared" ref="O69:O77" si="4">B69*M69</f>
         <v>0</v>
       </c>
       <c r="P69" s="32">
-        <f t="shared" ref="P69:P76" si="5">B69*N69</f>
+        <f t="shared" ref="P69:P77" si="5">B69*N69</f>
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A70" s="17">
         <v>63</v>
       </c>
@@ -4588,7 +4591,7 @@
         <v>0.307</v>
       </c>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A71">
         <v>64</v>
       </c>
@@ -4631,7 +4634,7 @@
         <v>1.32</v>
       </c>
     </row>
-    <row r="72" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A72" s="17">
         <v>65</v>
       </c>
@@ -4672,7 +4675,7 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A73">
         <v>66</v>
       </c>
@@ -4715,7 +4718,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A74" s="17">
         <v>67</v>
       </c>
@@ -4761,7 +4764,7 @@
         <v>0.39600000000000002</v>
       </c>
     </row>
-    <row r="75" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A75">
         <v>68</v>
       </c>
@@ -4779,98 +4782,124 @@
       <c r="M75" s="28"/>
       <c r="N75" s="28"/>
       <c r="O75" s="32">
+        <f t="shared" ref="O75" si="6">B75*M75</f>
+        <v>0</v>
+      </c>
+      <c r="P75" s="32">
+        <f t="shared" ref="P75" si="7">B75*N75</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.5">
+      <c r="A76">
+        <v>69</v>
+      </c>
+      <c r="B76" s="2">
+        <v>0</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D76" s="10" t="s">
+        <v>370</v>
+      </c>
+      <c r="J76" s="19"/>
+      <c r="L76"/>
+      <c r="M76" s="28"/>
+      <c r="N76" s="28"/>
+      <c r="O76" s="32">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="P75" s="32">
+      <c r="P76" s="32">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A76" s="17">
-        <v>69</v>
-      </c>
-      <c r="B76">
-        <v>1</v>
-      </c>
-      <c r="C76" t="s">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.5">
+      <c r="A77" s="17">
+        <v>70</v>
+      </c>
+      <c r="B77">
+        <v>1</v>
+      </c>
+      <c r="C77" t="s">
         <v>106</v>
       </c>
-      <c r="D76" t="s">
+      <c r="D77" t="s">
         <v>138</v>
       </c>
-      <c r="E76" t="s">
+      <c r="E77" t="s">
         <v>187</v>
       </c>
-      <c r="F76" t="s">
+      <c r="F77" t="s">
         <v>188</v>
       </c>
-      <c r="G76" t="s">
+      <c r="G77" t="s">
         <v>189</v>
       </c>
-      <c r="H76" t="s">
+      <c r="H77" t="s">
         <v>191</v>
       </c>
-      <c r="J76" s="36"/>
-      <c r="K76" t="s">
+      <c r="J77" s="36"/>
+      <c r="K77" t="s">
         <v>190</v>
       </c>
-      <c r="L76" s="13">
+      <c r="L77" s="13">
         <v>4300</v>
       </c>
-      <c r="M76">
+      <c r="M77">
         <v>0.27100000000000002</v>
       </c>
-      <c r="N76">
+      <c r="N77">
         <v>0.20499999999999999</v>
       </c>
-      <c r="O76">
+      <c r="O77">
         <f t="shared" si="4"/>
         <v>0.27100000000000002</v>
       </c>
-      <c r="P76">
+      <c r="P77">
         <f t="shared" si="5"/>
         <v>0.20499999999999999</v>
       </c>
     </row>
-    <row r="77" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.4">
-      <c r="M77" s="26"/>
-      <c r="N77" s="26"/>
-    </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="O78" s="1"/>
-    </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="O79" s="1">
-        <f>SUM(O3:O76)</f>
+    <row r="78" spans="1:16" s="6" customFormat="1" x14ac:dyDescent="0.5">
+      <c r="M78" s="26"/>
+      <c r="N78" s="26"/>
+    </row>
+    <row r="79" spans="1:16" x14ac:dyDescent="0.5">
+      <c r="O79" s="1"/>
+    </row>
+    <row r="80" spans="1:16" x14ac:dyDescent="0.5">
+      <c r="O80" s="1">
+        <f>SUM(O3:O77)</f>
         <v>57.314999999999998</v>
       </c>
-      <c r="P79" s="32">
-        <f>SUM(P3:P76)</f>
+      <c r="P80" s="32">
+        <f>SUM(P3:P77)</f>
         <v>42.715999999999994</v>
       </c>
     </row>
-    <row r="81" spans="4:16" x14ac:dyDescent="0.4">
-      <c r="O81" s="3"/>
-      <c r="P81" s="3"/>
-    </row>
-    <row r="83" spans="4:16" x14ac:dyDescent="0.4">
-      <c r="M83" s="1"/>
-      <c r="N83" s="1"/>
-      <c r="O83" s="1"/>
-    </row>
-    <row r="84" spans="4:16" x14ac:dyDescent="0.4">
+    <row r="82" spans="4:16" x14ac:dyDescent="0.5">
+      <c r="O82" s="3"/>
+      <c r="P82" s="3"/>
+    </row>
+    <row r="84" spans="4:16" x14ac:dyDescent="0.5">
       <c r="M84" s="1"/>
       <c r="N84" s="1"/>
       <c r="O84" s="1"/>
-      <c r="P84" s="1"/>
-    </row>
-    <row r="93" spans="4:16" x14ac:dyDescent="0.4">
-      <c r="D93" s="8"/>
-    </row>
-    <row r="94" spans="4:16" x14ac:dyDescent="0.4">
+    </row>
+    <row r="85" spans="4:16" x14ac:dyDescent="0.5">
+      <c r="M85" s="1"/>
+      <c r="N85" s="1"/>
+      <c r="O85" s="1"/>
+      <c r="P85" s="1"/>
+    </row>
+    <row r="94" spans="4:16" x14ac:dyDescent="0.5">
       <c r="D94" s="8"/>
+    </row>
+    <row r="95" spans="4:16" x14ac:dyDescent="0.5">
+      <c r="D95" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4887,22 +4916,22 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{559E5722-1C6B-4E42-89B4-3A44026BEFD4}">
-  <dimension ref="A1:R86"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" outlineLevelCol="1" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:R87"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.35" outlineLevelCol="1" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="4.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.3828125" customWidth="1"/>
-    <col min="3" max="3" width="31.3828125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="66.84375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.61328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.07421875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.4609375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.3828125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.921875" customWidth="1" outlineLevel="1"/>
-    <col min="10" max="18" width="10.921875" customWidth="1" outlineLevel="1"/>
+    <col min="1" max="1" width="4.3515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.3515625" customWidth="1"/>
+    <col min="3" max="3" width="31.3515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="66.8203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5859375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.05859375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.46875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.3515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.9375" customWidth="1" outlineLevel="1"/>
+    <col min="10" max="18" width="10.9375" customWidth="1" outlineLevel="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -4928,7 +4957,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A2">
         <v>1</v>
       </c>
@@ -4954,7 +4983,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A3">
         <v>2</v>
       </c>
@@ -4979,7 +5008,7 @@
       <c r="H3" s="7"/>
       <c r="I3" s="7"/>
     </row>
-    <row r="4" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A4">
         <v>3</v>
       </c>
@@ -5002,7 +5031,7 @@
         <v>805</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A5">
         <v>4</v>
       </c>
@@ -5025,7 +5054,7 @@
         <v>1210</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A6">
         <v>5</v>
       </c>
@@ -5048,7 +5077,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A7">
         <v>6</v>
       </c>
@@ -5071,7 +5100,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A8">
         <v>7</v>
       </c>
@@ -5094,7 +5123,7 @@
         <v>1206</v>
       </c>
     </row>
-    <row r="9" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A9">
         <v>8</v>
       </c>
@@ -5118,7 +5147,7 @@
       </c>
       <c r="H9" s="9"/>
     </row>
-    <row r="10" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A10">
         <v>9</v>
       </c>
@@ -5132,7 +5161,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A11">
         <v>10</v>
       </c>
@@ -5158,7 +5187,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A12">
         <v>11</v>
       </c>
@@ -5185,7 +5214,7 @@
       </c>
       <c r="I12" s="7"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A13">
         <v>12</v>
       </c>
@@ -5213,7 +5242,7 @@
       <c r="I13" s="7"/>
       <c r="J13" s="7"/>
     </row>
-    <row r="14" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:10" s="12" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A14">
         <v>13</v>
       </c>
@@ -5239,7 +5268,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A15">
         <v>14</v>
       </c>
@@ -5265,7 +5294,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A16">
         <v>15</v>
       </c>
@@ -5291,7 +5320,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A17">
         <v>16</v>
       </c>
@@ -5317,7 +5346,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A18">
         <v>17</v>
       </c>
@@ -5343,7 +5372,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A19">
         <v>18</v>
       </c>
@@ -5369,7 +5398,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="20" spans="1:12" s="12" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:12" s="12" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A20">
         <v>19</v>
       </c>
@@ -5395,7 +5424,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A21">
         <v>20</v>
       </c>
@@ -5421,7 +5450,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A22">
         <v>21</v>
       </c>
@@ -5447,7 +5476,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A23">
         <v>22</v>
       </c>
@@ -5473,7 +5502,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A24">
         <v>23</v>
       </c>
@@ -5499,7 +5528,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A25">
         <v>24</v>
       </c>
@@ -5525,7 +5554,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A26">
         <v>25</v>
       </c>
@@ -5551,7 +5580,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="27" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A27">
         <v>26</v>
       </c>
@@ -5566,7 +5595,7 @@
       </c>
       <c r="G27" s="10"/>
     </row>
-    <row r="28" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A28">
         <v>27</v>
       </c>
@@ -5580,7 +5609,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A29">
         <v>28</v>
       </c>
@@ -5606,7 +5635,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A30">
         <v>29</v>
       </c>
@@ -5635,7 +5664,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A31">
         <v>30</v>
       </c>
@@ -5661,7 +5690,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A32">
         <v>31</v>
       </c>
@@ -5687,7 +5716,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A33">
         <v>32</v>
       </c>
@@ -5713,7 +5742,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A34">
         <v>33</v>
       </c>
@@ -5739,7 +5768,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="35" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A35">
         <v>34</v>
       </c>
@@ -5765,7 +5794,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A36">
         <v>35</v>
       </c>
@@ -5788,7 +5817,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A37">
         <v>36</v>
       </c>
@@ -5812,7 +5841,7 @@
       </c>
       <c r="I37" s="7"/>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A38">
         <v>37</v>
       </c>
@@ -5837,7 +5866,7 @@
       <c r="H38" s="7"/>
       <c r="I38" s="7"/>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A39">
         <v>38</v>
       </c>
@@ -5862,7 +5891,7 @@
       <c r="H39" s="9"/>
       <c r="I39" s="34"/>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A40">
         <v>39</v>
       </c>
@@ -5885,7 +5914,7 @@
       <c r="H40" s="7"/>
       <c r="I40" s="7"/>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A41">
         <v>40</v>
       </c>
@@ -5910,7 +5939,7 @@
       <c r="H41" s="7"/>
       <c r="I41" s="7"/>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A42">
         <v>41</v>
       </c>
@@ -5935,7 +5964,7 @@
       <c r="H42" s="7"/>
       <c r="I42" s="7"/>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A43">
         <v>42</v>
       </c>
@@ -5959,7 +5988,7 @@
       </c>
       <c r="I43" s="7"/>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A44">
         <v>43</v>
       </c>
@@ -5983,7 +6012,7 @@
       </c>
       <c r="I44" s="7"/>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A45">
         <v>44</v>
       </c>
@@ -6007,7 +6036,7 @@
       </c>
       <c r="I45" s="7"/>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A46">
         <v>46</v>
       </c>
@@ -6031,7 +6060,7 @@
       </c>
       <c r="I46" s="7"/>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A47">
         <v>47</v>
       </c>
@@ -6057,7 +6086,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A48">
         <v>48</v>
       </c>
@@ -6083,7 +6112,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A49">
         <v>49</v>
       </c>
@@ -6109,7 +6138,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="50" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A50">
         <v>50</v>
       </c>
@@ -6135,7 +6164,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A51">
         <v>51</v>
       </c>
@@ -6159,7 +6188,7 @@
       </c>
       <c r="H51" s="7"/>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A52">
         <v>52</v>
       </c>
@@ -6183,7 +6212,7 @@
       </c>
       <c r="H52" s="7"/>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A53">
         <v>53</v>
       </c>
@@ -6207,7 +6236,7 @@
       </c>
       <c r="H53" s="7"/>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A54">
         <v>54</v>
       </c>
@@ -6233,7 +6262,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="55" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A55">
         <v>55</v>
       </c>
@@ -6259,7 +6288,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="56" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A56">
         <v>56</v>
       </c>
@@ -6285,7 +6314,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="57" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A57" s="17">
         <v>57</v>
       </c>
@@ -6308,7 +6337,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="58" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A58" s="17">
         <v>58</v>
       </c>
@@ -6331,7 +6360,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A59" s="17">
         <v>59</v>
       </c>
@@ -6357,7 +6386,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A60" s="17">
         <v>60</v>
       </c>
@@ -6378,7 +6407,7 @@
       </c>
       <c r="G60" s="7"/>
     </row>
-    <row r="61" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A61" s="17">
         <v>61</v>
       </c>
@@ -6401,7 +6430,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A62" s="17">
         <v>62</v>
       </c>
@@ -6418,7 +6447,7 @@
       <c r="F62" s="2"/>
       <c r="G62" s="2"/>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A63" s="17">
         <v>63</v>
       </c>
@@ -6441,7 +6470,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="64" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A64" s="17">
         <v>64</v>
       </c>
@@ -6462,7 +6491,7 @@
       </c>
       <c r="G64"/>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A65" s="17">
         <v>65</v>
       </c>
@@ -6483,7 +6512,7 @@
       </c>
       <c r="G65" s="7"/>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A66" s="17">
         <v>66</v>
       </c>
@@ -6503,7 +6532,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.5">
       <c r="A67" s="17">
         <v>67</v>
       </c>
@@ -6526,7 +6555,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A68" s="17">
         <v>68</v>
       </c>
@@ -6543,34 +6572,51 @@
       <c r="F68" s="2"/>
       <c r="G68" s="2"/>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.5">
       <c r="A69" s="17">
         <v>69</v>
       </c>
-      <c r="B69">
-        <v>1</v>
-      </c>
-      <c r="C69" s="9" t="s">
+      <c r="B69" s="2">
+        <v>0</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D69" s="10" t="s">
+        <v>370</v>
+      </c>
+      <c r="E69" s="2"/>
+      <c r="F69" s="2"/>
+      <c r="G69" s="2"/>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.5">
+      <c r="A70" s="17">
+        <v>70</v>
+      </c>
+      <c r="B70">
+        <v>1</v>
+      </c>
+      <c r="C70" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="D69" t="s">
+      <c r="D70" t="s">
         <v>138</v>
       </c>
-      <c r="E69" t="s">
+      <c r="E70" t="s">
         <v>187</v>
       </c>
-      <c r="F69" t="s">
+      <c r="F70" t="s">
         <v>188</v>
       </c>
-      <c r="G69" t="s">
+      <c r="G70" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="85" spans="4:4" x14ac:dyDescent="0.4">
-      <c r="D85" s="8"/>
-    </row>
-    <row r="86" spans="4:4" x14ac:dyDescent="0.4">
+    <row r="86" spans="4:4" x14ac:dyDescent="0.5">
       <c r="D86" s="8"/>
+    </row>
+    <row r="87" spans="4:4" x14ac:dyDescent="0.5">
+      <c r="D87" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>